<commit_message>
Status coming in benficiries forms
</commit_message>
<xml_diff>
--- a/SukrtyaQuestion.filled.xlsx
+++ b/SukrtyaQuestion.filled.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DIGITCore\sukrtya-siwan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2CD1F7-0B71-451C-B113-0074BBF4A147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03233F56-4B8C-4B56-B8A0-DD39BDC89A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="129">
   <si>
     <t>faQID</t>
   </si>
@@ -152,9 +152,6 @@
     <t xml:space="preserve">Place of 1st ANC </t>
   </si>
   <si>
-    <t>FORM1</t>
-  </si>
-  <si>
     <t>BP:  Systolic/ diastolic</t>
   </si>
   <si>
@@ -405,13 +402,22 @@
   </si>
   <si>
     <t>DeliveryDetails</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>DEMO</t>
+  </si>
+  <si>
+    <t>DEMO1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -432,8 +438,14 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -473,6 +485,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE699"/>
+        <bgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
@@ -638,7 +662,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -737,7 +761,24 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1072,13 +1113,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P89"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="24.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.88671875" style="30" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" style="30" bestFit="1" customWidth="1"/>
@@ -1294,7 +1335,7 @@
       <c r="A11" s="6">
         <v>10</v>
       </c>
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="5" t="s">
@@ -1330,7 +1371,7 @@
       <c r="A12" s="6">
         <v>11</v>
       </c>
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -1366,7 +1407,7 @@
       <c r="A13" s="6">
         <v>12</v>
       </c>
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -1402,7 +1443,7 @@
       <c r="A14" s="6">
         <v>13</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -1438,7 +1479,7 @@
       <c r="A15" s="6">
         <v>14</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="5" t="s">
@@ -1474,7 +1515,7 @@
       <c r="A16" s="6">
         <v>15</v>
       </c>
-      <c r="B16" s="48" t="s">
+      <c r="B16" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -1506,11 +1547,11 @@
       </c>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -1542,11 +1583,11 @@
       </c>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>17</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="47" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -1576,7 +1617,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -1610,7 +1651,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -1646,7 +1687,7 @@
       </c>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -1681,14 +1722,8 @@
         <v>45292</v>
       </c>
       <c r="L21" s="14"/>
-      <c r="O21" t="s">
-        <v>37</v>
-      </c>
-      <c r="P21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -1696,13 +1731,13 @@
         <v>37</v>
       </c>
       <c r="C22" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="F22" s="33" t="s">
         <v>21</v>
@@ -1723,14 +1758,8 @@
         <v>0</v>
       </c>
       <c r="L22" s="14"/>
-      <c r="O22" t="s">
-        <v>45</v>
-      </c>
-      <c r="P22" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -1738,7 +1767,7 @@
         <v>37</v>
       </c>
       <c r="C23" s="40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>21</v>
@@ -1765,14 +1794,8 @@
         <v>0</v>
       </c>
       <c r="L23" s="14"/>
-      <c r="O23" t="s">
-        <v>47</v>
-      </c>
-      <c r="P23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -1780,23 +1803,23 @@
         <v>37</v>
       </c>
       <c r="C24" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E24" s="10" t="s">
+      <c r="F24" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F24" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="I24" s="6">
         <v>0</v>
       </c>
@@ -1807,14 +1830,8 @@
         <v>21</v>
       </c>
       <c r="L24" s="14"/>
-      <c r="O24" t="s">
-        <v>51</v>
-      </c>
-      <c r="P24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -1822,13 +1839,13 @@
         <v>37</v>
       </c>
       <c r="C25" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="F25" s="33">
         <v>2</v>
@@ -1837,7 +1854,7 @@
         <v>29</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I25" s="6">
         <v>1</v>
@@ -1850,7 +1867,7 @@
       </c>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -1858,14 +1875,14 @@
         <v>37</v>
       </c>
       <c r="C26" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>55</v>
-      </c>
       <c r="F26" s="33" t="s">
         <v>21</v>
       </c>
@@ -1873,7 +1890,7 @@
         <v>21</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I26" s="6">
         <v>1</v>
@@ -1886,7 +1903,7 @@
       </c>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -1894,13 +1911,13 @@
         <v>37</v>
       </c>
       <c r="C27" s="40" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F27" s="33">
         <v>2</v>
@@ -1909,7 +1926,7 @@
         <v>29</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I27" s="6">
         <v>1</v>
@@ -1922,7 +1939,7 @@
       </c>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -1930,7 +1947,7 @@
         <v>37</v>
       </c>
       <c r="C28" s="40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>21</v>
@@ -1958,7 +1975,7 @@
       </c>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -1966,7 +1983,7 @@
         <v>37</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>21</v>
@@ -1994,7 +2011,7 @@
       </c>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -2002,7 +2019,7 @@
         <v>37</v>
       </c>
       <c r="C30" s="41" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>21</v>
@@ -2030,15 +2047,15 @@
       </c>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>30</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C31" s="41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>21</v>
@@ -2061,18 +2078,18 @@
       <c r="J31" s="34"/>
       <c r="K31" s="34"/>
       <c r="L31" s="14" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="6">
         <v>31</v>
       </c>
       <c r="B32" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C32" s="41" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>21</v>
@@ -2105,10 +2122,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33" s="41" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>21</v>
@@ -2141,16 +2158,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C34" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="F34" s="33" t="s">
         <v>21</v>
@@ -2177,10 +2194,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="41" t="s">
         <v>45</v>
-      </c>
-      <c r="C35" s="41" t="s">
-        <v>46</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>21</v>
@@ -2213,25 +2230,25 @@
         <v>35</v>
       </c>
       <c r="B36" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C36" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D36" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E36" s="10" t="s">
+      <c r="F36" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="F36" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="I36" s="6">
         <v>0</v>
@@ -2249,16 +2266,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C37" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="F37" s="33">
         <v>2</v>
@@ -2267,7 +2284,7 @@
         <v>41</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I37" s="6">
         <v>1</v>
@@ -2285,17 +2302,17 @@
         <v>37</v>
       </c>
       <c r="B38" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C38" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E38" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>55</v>
-      </c>
       <c r="F38" s="33" t="s">
         <v>21</v>
       </c>
@@ -2303,7 +2320,7 @@
         <v>21</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I38" s="6">
         <v>1</v>
@@ -2321,16 +2338,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C39" s="41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F39" s="33">
         <v>2</v>
@@ -2339,7 +2356,7 @@
         <v>41</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I39" s="6">
         <v>1</v>
@@ -2357,10 +2374,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C40" s="41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>21</v>
@@ -2393,10 +2410,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C41" s="41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>21</v>
@@ -2429,10 +2446,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C42" s="42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>21</v>
@@ -2465,10 +2482,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C43" s="42" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>21</v>
@@ -2491,7 +2508,7 @@
       <c r="J43" s="34"/>
       <c r="K43" s="34"/>
       <c r="L43" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
@@ -2499,10 +2516,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C44" s="42" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>21</v>
@@ -2535,10 +2552,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C45" s="42" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>21</v>
@@ -2571,16 +2588,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C46" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="F46" s="33" t="s">
         <v>21</v>
@@ -2607,10 +2624,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C47" s="42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>21</v>
@@ -2643,25 +2660,25 @@
         <v>47</v>
       </c>
       <c r="B48" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="C48" s="42" t="s">
+      <c r="D48" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D48" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E48" s="10" t="s">
+      <c r="F48" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G48" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H48" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="F48" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G48" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="H48" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="I48" s="6">
         <v>0</v>
@@ -2679,16 +2696,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C49" s="42" t="s">
+        <v>51</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E49" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="F49" s="33">
         <v>2</v>
@@ -2697,7 +2714,7 @@
         <v>53</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I49" s="6">
         <v>1</v>
@@ -2715,16 +2732,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C50" s="42" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F50" s="33" t="s">
         <v>21</v>
@@ -2733,7 +2750,7 @@
         <v>21</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I50" s="6">
         <v>1</v>
@@ -2751,16 +2768,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C51" s="42" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F51" s="33">
         <v>2</v>
@@ -2769,7 +2786,7 @@
         <v>53</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I51" s="6">
         <v>1</v>
@@ -2787,10 +2804,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C52" s="42" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>21</v>
@@ -2823,10 +2840,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C53" s="42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>21</v>
@@ -2859,10 +2876,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C54" s="43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>21</v>
@@ -2895,10 +2912,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C55" s="43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>21</v>
@@ -2921,7 +2938,7 @@
       <c r="J55" s="34"/>
       <c r="K55" s="34"/>
       <c r="L55" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
@@ -2929,10 +2946,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C56" s="43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>21</v>
@@ -2965,10 +2982,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C57" s="43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>21</v>
@@ -3001,16 +3018,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C58" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E58" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="F58" s="33" t="s">
         <v>21</v>
@@ -3037,10 +3054,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C59" s="43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>21</v>
@@ -3073,25 +3090,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C60" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E60" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D60" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E60" s="10" t="s">
+      <c r="F60" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G60" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H60" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="F60" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="G60" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="H60" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="I60" s="6">
         <v>0</v>
@@ -3109,16 +3126,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="47" t="s">
+        <v>50</v>
+      </c>
+      <c r="C61" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="C61" s="43" t="s">
+      <c r="D61" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E61" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="F61" s="33">
         <v>2</v>
@@ -3127,7 +3144,7 @@
         <v>65</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I61" s="6">
         <v>1</v>
@@ -3145,16 +3162,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C62" s="43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F62" s="33" t="s">
         <v>21</v>
@@ -3163,7 +3180,7 @@
         <v>21</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I62" s="6">
         <v>1</v>
@@ -3181,16 +3198,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C63" s="43" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F63" s="33">
         <v>2</v>
@@ -3199,7 +3216,7 @@
         <v>65</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I63" s="6">
         <v>1</v>
@@ -3217,10 +3234,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C64" s="43" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>21</v>
@@ -3253,10 +3270,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C65" s="43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>21</v>
@@ -3289,10 +3306,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C66" s="41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>21</v>
@@ -3325,16 +3342,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C67" s="41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F67" s="33" t="s">
         <v>21</v>
@@ -3343,7 +3360,7 @@
         <v>21</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I67" s="6">
         <v>1</v>
@@ -3361,16 +3378,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C68" s="41" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F68" s="33" t="s">
         <v>21</v>
@@ -3379,7 +3396,7 @@
         <v>21</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I68" s="6">
         <v>1</v>
@@ -3397,16 +3414,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C69" s="41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F69" s="33" t="s">
         <v>21</v>
@@ -3415,7 +3432,7 @@
         <v>21</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I69" s="6">
         <v>0</v>
@@ -3433,16 +3450,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C70" s="41" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F70" s="33" t="s">
         <v>21</v>
@@ -3451,7 +3468,7 @@
         <v>21</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I70" s="6">
         <v>0</v>
@@ -3469,16 +3486,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C71" s="41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F71" s="33" t="s">
         <v>21</v>
@@ -3487,7 +3504,7 @@
         <v>21</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I71" s="6">
         <v>1</v>
@@ -3505,10 +3522,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C72" s="41" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>21</v>
@@ -3541,16 +3558,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C73" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E73" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="F73" s="33">
         <v>22</v>
@@ -3559,7 +3576,7 @@
         <v>88</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I73" s="6">
         <v>1</v>
@@ -3577,16 +3594,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C74" s="41" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F74" s="33" t="s">
         <v>21</v>
@@ -3595,7 +3612,7 @@
         <v>21</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I74" s="6">
         <v>1</v>
@@ -3613,10 +3630,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C75" s="41" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>21</v>
@@ -3649,16 +3666,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C76" s="41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F76" s="33" t="s">
         <v>21</v>
@@ -3667,7 +3684,7 @@
         <v>21</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I76" s="6">
         <v>1</v>
@@ -3685,10 +3702,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C77" s="41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>21</v>
@@ -3721,16 +3738,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C78" s="41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F78" s="33" t="s">
         <v>21</v>
@@ -3739,7 +3756,7 @@
         <v>21</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I78" s="6">
         <v>1</v>
@@ -3757,16 +3774,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C79" s="41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F79" s="33" t="s">
         <v>21</v>
@@ -3775,7 +3792,7 @@
         <v>21</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I79" s="6">
         <v>1</v>
@@ -3793,16 +3810,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C80" s="41" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F80" s="33">
         <v>2</v>
@@ -3811,7 +3828,7 @@
         <v>81</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I80" s="6">
         <v>1</v>
@@ -3829,16 +3846,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C81" s="41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F81" s="33" t="s">
         <v>21</v>
@@ -3847,7 +3864,7 @@
         <v>21</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I81" s="6">
         <v>0</v>
@@ -3865,16 +3882,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C82" s="44" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F82" s="33" t="s">
         <v>21</v>
@@ -3883,7 +3900,7 @@
         <v>21</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I82" s="6">
         <v>1</v>
@@ -3901,16 +3918,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C83" s="44" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F83" s="33" t="s">
         <v>21</v>
@@ -3919,7 +3936,7 @@
         <v>21</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I83" s="6">
         <v>0</v>
@@ -3937,16 +3954,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C84" s="44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F84" s="33" t="s">
         <v>21</v>
@@ -3955,7 +3972,7 @@
         <v>21</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I84" s="6">
         <v>0</v>
@@ -3973,16 +3990,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C85" s="44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F85" s="33" t="s">
         <v>21</v>
@@ -3991,7 +4008,7 @@
         <v>21</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I85" s="6">
         <v>0</v>
@@ -4009,16 +4026,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C86" s="44" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F86" s="33" t="s">
         <v>21</v>
@@ -4027,7 +4044,7 @@
         <v>21</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I86" s="6">
         <v>0</v>
@@ -4045,16 +4062,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C87" s="44" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F87" s="33" t="s">
         <v>21</v>
@@ -4063,7 +4080,7 @@
         <v>21</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I87" s="6">
         <v>0</v>
@@ -4081,16 +4098,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C88" s="44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>21</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F88" s="33" t="s">
         <v>21</v>
@@ -4099,7 +4116,7 @@
         <v>21</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I88" s="6">
         <v>0</v>
@@ -4117,7 +4134,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C89" s="45" t="s">
         <v>11</v>
@@ -4146,8 +4163,907 @@
       </c>
       <c r="L89" s="14"/>
     </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A90" s="48">
+        <v>89</v>
+      </c>
+      <c r="B90" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C90" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="D90" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E90" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F90" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G90" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H90" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="I90" s="48">
+        <v>1</v>
+      </c>
+      <c r="J90" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="K90" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="L90" s="54"/>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A91" s="48">
+        <v>90</v>
+      </c>
+      <c r="B91" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C91" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="D91" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E91" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F91" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G91" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H91" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="I91" s="48">
+        <v>0</v>
+      </c>
+      <c r="J91" s="53">
+        <v>9999999999</v>
+      </c>
+      <c r="K91" s="53">
+        <v>0</v>
+      </c>
+      <c r="L91" s="54"/>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A92" s="48">
+        <v>91</v>
+      </c>
+      <c r="B92" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C92" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="D92" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E92" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F92" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G92" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H92" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="I92" s="48">
+        <v>0</v>
+      </c>
+      <c r="J92" s="53">
+        <v>9999999999</v>
+      </c>
+      <c r="K92" s="53">
+        <v>0</v>
+      </c>
+      <c r="L92" s="54"/>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A93" s="48">
+        <v>92</v>
+      </c>
+      <c r="B93" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C93" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="D93" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E93" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F93" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G93" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H93" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="I93" s="48">
+        <v>0</v>
+      </c>
+      <c r="J93" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="K93" s="55">
+        <v>45292</v>
+      </c>
+      <c r="L93" s="54"/>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A94" s="48">
+        <v>93</v>
+      </c>
+      <c r="B94" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C94" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="D94" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E94" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F94" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G94" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H94" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="I94" s="48">
+        <v>0</v>
+      </c>
+      <c r="J94" s="53">
+        <v>9999999999</v>
+      </c>
+      <c r="K94" s="53">
+        <v>0</v>
+      </c>
+      <c r="L94" s="54"/>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A95" s="48">
+        <v>94</v>
+      </c>
+      <c r="B95" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C95" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="D95" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E95" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F95" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G95" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H95" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="I95" s="48">
+        <v>1</v>
+      </c>
+      <c r="J95" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="K95" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="L95" s="54"/>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A96" s="48">
+        <v>95</v>
+      </c>
+      <c r="B96" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C96" s="50" t="s">
+        <v>32</v>
+      </c>
+      <c r="D96" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E96" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F96" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G96" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H96" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="I96" s="48">
+        <v>1</v>
+      </c>
+      <c r="J96" s="53">
+        <v>9999999999</v>
+      </c>
+      <c r="K96" s="53">
+        <v>0</v>
+      </c>
+      <c r="L96" s="54"/>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A97" s="48">
+        <v>96</v>
+      </c>
+      <c r="B97" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C97" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="D97" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E97" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F97" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G97" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H97" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="I97" s="48">
+        <v>1</v>
+      </c>
+      <c r="J97" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="K97" s="55">
+        <v>45292</v>
+      </c>
+      <c r="L97" s="54"/>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A98" s="48">
+        <v>97</v>
+      </c>
+      <c r="B98" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="C98" s="50" t="s">
+        <v>34</v>
+      </c>
+      <c r="D98" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E98" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F98" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G98" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="H98" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="I98" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="J98" s="55"/>
+      <c r="K98" s="55"/>
+      <c r="L98" s="54" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A99" s="6">
+        <v>65</v>
+      </c>
+      <c r="B99" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C99" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F99" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G99" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I99" s="6">
+        <v>0</v>
+      </c>
+      <c r="J99" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="K99" s="34">
+        <v>45292</v>
+      </c>
+      <c r="L99" s="14"/>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A100" s="6">
+        <v>66</v>
+      </c>
+      <c r="B100" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C100" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E100" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F100" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G100" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I100" s="6">
+        <v>1</v>
+      </c>
+      <c r="J100" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K100" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L100" s="14"/>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A101" s="6">
+        <v>67</v>
+      </c>
+      <c r="B101" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C101" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E101" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F101" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G101" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I101" s="6">
+        <v>1</v>
+      </c>
+      <c r="J101" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K101" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L101" s="14"/>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A102" s="6">
+        <v>68</v>
+      </c>
+      <c r="B102" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C102" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E102" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F102" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G102" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H102" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I102" s="6">
+        <v>0</v>
+      </c>
+      <c r="J102" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K102" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L102" s="14"/>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A103" s="6">
+        <v>69</v>
+      </c>
+      <c r="B103" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C103" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E103" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F103" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G103" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H103" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I103" s="6">
+        <v>0</v>
+      </c>
+      <c r="J103" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K103" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L103" s="14"/>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A104" s="6">
+        <v>70</v>
+      </c>
+      <c r="B104" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C104" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E104" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F104" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G104" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H104" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I104" s="6">
+        <v>1</v>
+      </c>
+      <c r="J104" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K104" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L104" s="14"/>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A105" s="6">
+        <v>71</v>
+      </c>
+      <c r="B105" s="47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C105" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F105" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G105" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I105" s="6">
+        <v>1</v>
+      </c>
+      <c r="J105" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="K105" s="34">
+        <v>45292</v>
+      </c>
+      <c r="L105" s="14"/>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A106" s="6">
+        <v>72</v>
+      </c>
+      <c r="B106" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C106" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E106" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F106" s="33">
+        <v>22</v>
+      </c>
+      <c r="G106" s="33">
+        <v>88</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I106" s="6">
+        <v>1</v>
+      </c>
+      <c r="J106" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K106" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L106" s="14"/>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A107" s="6">
+        <v>73</v>
+      </c>
+      <c r="B107" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C107" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E107" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F107" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G107" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I107" s="6">
+        <v>1</v>
+      </c>
+      <c r="J107" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="K107" s="34">
+        <v>45292</v>
+      </c>
+      <c r="L107" s="14"/>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A108" s="6">
+        <v>74</v>
+      </c>
+      <c r="B108" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C108" s="41" t="s">
+        <v>82</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E108" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F108" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G108" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H108" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I108" s="6">
+        <v>0</v>
+      </c>
+      <c r="J108" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="K108" s="34">
+        <v>45292</v>
+      </c>
+      <c r="L108" s="14"/>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A109" s="6">
+        <v>75</v>
+      </c>
+      <c r="B109" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C109" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E109" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F109" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G109" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H109" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I109" s="6">
+        <v>1</v>
+      </c>
+      <c r="J109" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K109" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L109" s="14"/>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A110" s="6">
+        <v>76</v>
+      </c>
+      <c r="B110" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C110" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E110" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F110" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H110" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I110" s="6">
+        <v>1</v>
+      </c>
+      <c r="J110" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K110" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L110" s="14"/>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A111" s="6">
+        <v>77</v>
+      </c>
+      <c r="B111" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C111" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="D111" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E111" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F111" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G111" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H111" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I111" s="6">
+        <v>1</v>
+      </c>
+      <c r="J111" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K111" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L111" s="14"/>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A112" s="6">
+        <v>78</v>
+      </c>
+      <c r="B112" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C112" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E112" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F112" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G112" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H112" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I112" s="6">
+        <v>1</v>
+      </c>
+      <c r="J112" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K112" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L112" s="14"/>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A113" s="6">
+        <v>79</v>
+      </c>
+      <c r="B113" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C113" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E113" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F113" s="33">
+        <v>2</v>
+      </c>
+      <c r="G113" s="33">
+        <v>81</v>
+      </c>
+      <c r="H113" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I113" s="6">
+        <v>1</v>
+      </c>
+      <c r="J113" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K113" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L113" s="14"/>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A114" s="6">
+        <v>80</v>
+      </c>
+      <c r="B114" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="C114" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E114" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F114" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G114" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H114" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I114" s="6">
+        <v>0</v>
+      </c>
+      <c r="J114" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="K114" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L114" s="14"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
@@ -4164,13 +5080,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -4178,7 +5094,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C2" s="2"/>
     </row>
@@ -4187,7 +5103,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -4196,7 +5112,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C4" s="2"/>
     </row>
@@ -4205,7 +5121,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -4214,7 +5130,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" s="2"/>
     </row>
@@ -4223,7 +5139,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -4232,7 +5148,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" s="2"/>
     </row>
@@ -4241,7 +5157,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C9" s="2"/>
     </row>
@@ -4250,7 +5166,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C10" s="2"/>
     </row>
@@ -4259,7 +5175,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C11" s="2"/>
     </row>
@@ -4268,7 +5184,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C12" s="2"/>
     </row>
@@ -4277,7 +5193,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C13" s="2"/>
     </row>
@@ -4286,7 +5202,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -4295,7 +5211,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C15" s="2"/>
     </row>
@@ -4304,7 +5220,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C16" s="2"/>
     </row>
@@ -4313,7 +5229,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C17" s="2"/>
     </row>
@@ -4322,7 +5238,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C18" s="2"/>
     </row>
@@ -4331,7 +5247,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C19" s="2"/>
     </row>
@@ -4340,7 +5256,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C20" s="2"/>
     </row>
@@ -4349,7 +5265,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C21" s="2"/>
     </row>
@@ -4358,7 +5274,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C22" s="2"/>
     </row>
@@ -4367,7 +5283,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C23" s="2"/>
     </row>
@@ -4376,7 +5292,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C24" s="2"/>
     </row>
@@ -4385,7 +5301,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C25" s="2"/>
     </row>
@@ -4394,7 +5310,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C26" s="2"/>
     </row>

</xml_diff>